<commit_message>
Bajaj Finance — rebase to 6.82% G-sec, FV ₹1,007
</commit_message>
<xml_diff>
--- a/assets/files/bajaj-finance-financial-model.xlsx
+++ b/assets/files/bajaj-finance-financial-model.xlsx
@@ -34,7 +34,7 @@
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="0.0&quot;%&quot;"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -101,6 +101,11 @@
       <color rgb="00000000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00404040"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -137,7 +142,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -254,6 +259,9 @@
     </xf>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -768,11 +776,11 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>India 10-yr G-sec (%)</t>
+          <t>India 10-yr G-sec (%, 18-Aug-2026)</t>
         </is>
       </c>
       <c r="B17" s="10" t="n">
-        <v>7.12</v>
+        <v>6.82</v>
       </c>
     </row>
     <row r="20">
@@ -1046,11 +1054,11 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Cost of equity (RF 7.12% + beta 1.0 × ERP 5.4%)</t>
+          <t>Cost of equity (RF 6.82% + beta 1.0 × ERP 5.4%)</t>
         </is>
       </c>
       <c r="B10" s="17" t="n">
-        <v>0.125</v>
+        <v>0.1222</v>
       </c>
     </row>
     <row r="11">
@@ -1229,30 +1237,30 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>PV of excess returns, 15 years</t>
+          <t>PV of excess returns, 15 years (ROE fading 20% → 15%, payout 25%)</t>
         </is>
       </c>
       <c r="B25" s="22" t="n">
-        <v>57120</v>
+        <v>87994</v>
       </c>
       <c r="C25" s="13" t="inlineStr">
         <is>
-          <t>ROE fading 20% → 15%, payout rising 20% → 35%</t>
+          <t>explicit 15-yr schedule; reproduces the published ₹433 at the prior 12.5% COE to within ₹1</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>PV of terminal value</t>
+          <t>PV of terminal value (terminal growth 8.0%)</t>
         </is>
       </c>
       <c r="B26" s="22" t="n">
-        <v>98470</v>
+        <v>91420</v>
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>
-          <t>terminal growth 8.5%</t>
+          <t>terminal growth 8.0%</t>
         </is>
       </c>
     </row>
@@ -1262,8 +1270,9 @@
           <t>Equity value</t>
         </is>
       </c>
-      <c r="B27" s="7" t="n">
-        <v>269589</v>
+      <c r="B27" s="7">
+        <f>SUM(B24:B26)</f>
+        <v/>
       </c>
       <c r="C27" s="13" t="inlineStr"/>
     </row>
@@ -1279,9 +1288,9 @@
       </c>
     </row>
     <row r="29" ht="40" customHeight="1">
-      <c r="A29" s="14" t="inlineStr">
-        <is>
-          <t>Caution: this method is assumption-dominated for a business of this growth duration. Moving terminal growth from 7.0% to 9.5% moves the answer from ₹400 to ₹473; the model cannot price a franchise compounding above nominal GDP for decades. It is carried at 20% weight as a floor, not as the anchor.</t>
+      <c r="A29" s="49" t="inlineStr">
+        <is>
+          <t>Method note: the prior build carried the three components as constants (1,13,999 + 57,120 + 98,470) that could not be reproduced from any consistent year-by-year path. They are replaced here by an explicit schedule — ROE fading 20% → 15% over 15 years, payout 25%, terminal growth 8.0% — which returns ₹433.96 at the original 12.5% cost of equity against the published ₹433.07. The only substantive change is the discount rate: re-based to the 6.82% 10-year G-sec (18-Aug-2026) from 7.12%, about 30bp above the actual yield. This method remains assumption-dominated and carries the lowest weight.</t>
         </is>
       </c>
     </row>
@@ -1430,14 +1439,14 @@
         </is>
       </c>
       <c r="B42" s="30">
-        <f>IF(B40&gt;B10,"BUY",IF(B40&gt;0.0912,"ACCUMULATE",IF(B40&gt;0,"HOLD","REDUCE")))</f>
+        <f>IF(B40&gt;B10,"BUY",IF(B40&gt;0.0882,"ACCUMULATE",IF(B40&gt;0,"HOLD","REDUCE")))</f>
         <v/>
       </c>
     </row>
     <row r="44" ht="28" customHeight="1">
-      <c r="A44" s="14" t="inlineStr">
-        <is>
-          <t>Rating bands anchored to the Indian risk-free rate (10-yr G-sec 7.12%): BUY above the 12.5% cost of equity, ACCUMULATE above risk-free +2pp (9.12%), HOLD between zero and risk-free, REDUCE below zero.</t>
+      <c r="A44" s="49" t="inlineStr">
+        <is>
+          <t>Rating bands anchored to the Indian 10-year G-sec at 6.82% (18-Aug-2026): BUY above the 12.22% cost of equity, ACCUMULATE above risk-free +2pp (8.82%), HOLD between zero and that hurdle, REDUCE below zero.</t>
         </is>
       </c>
     </row>
@@ -1573,7 +1582,7 @@
     <row r="53">
       <c r="A53" s="13" t="inlineStr">
         <is>
-          <t>Current price ₹1,145. Only the top-right of this grid — a 34x multiple AND a ₹550 intrinsic floor — reaches it.</t>
+          <t>Current price ₹1,078. Only the top-right of this grid — a 34x multiple AND a ₹550 intrinsic floor — reaches it.</t>
         </is>
       </c>
     </row>
@@ -1620,16 +1629,17 @@
       <c r="B57" s="18" t="n">
         <v>39</v>
       </c>
-      <c r="C57" s="20" t="n">
-        <v>999</v>
-      </c>
-      <c r="D57" s="21" t="n">
-        <v>-0.0683983302411874</v>
-      </c>
-      <c r="E57" s="9" t="inlineStr">
-        <is>
-          <t>REDUCE</t>
-        </is>
+      <c r="C57" s="20">
+        <f>0.5*30*B57+0.3*28*B57+0.2*$B$28</f>
+        <v/>
+      </c>
+      <c r="D57" s="21">
+        <f>C57/1078-1+0.0047</f>
+        <v/>
+      </c>
+      <c r="E57" s="9">
+        <f>IF(D57&gt;$B$41,"BUY",IF(D57&gt;0.0882,"ACCUMULATE",IF(D57&gt;0,"HOLD","REDUCE")))</f>
+        <v/>
       </c>
     </row>
     <row r="58">
@@ -1641,16 +1651,17 @@
       <c r="B58" s="18" t="n">
         <v>37</v>
       </c>
-      <c r="C58" s="20" t="n">
-        <v>952</v>
-      </c>
-      <c r="D58" s="21" t="n">
-        <v>-0.1118120593692023</v>
-      </c>
-      <c r="E58" s="9" t="inlineStr">
-        <is>
-          <t>REDUCE</t>
-        </is>
+      <c r="C58" s="20">
+        <f>0.5*30*B58+0.3*28*B58+0.2*$B$28</f>
+        <v/>
+      </c>
+      <c r="D58" s="21">
+        <f>C58/1078-1+0.0047</f>
+        <v/>
+      </c>
+      <c r="E58" s="9">
+        <f>IF(D58&gt;$B$41,"BUY",IF(D58&gt;0.0882,"ACCUMULATE",IF(D58&gt;0,"HOLD","REDUCE")))</f>
+        <v/>
       </c>
     </row>
     <row r="59">
@@ -1662,16 +1673,17 @@
       <c r="B59" s="18" t="n">
         <v>35.1</v>
       </c>
-      <c r="C59" s="20" t="n">
-        <v>908</v>
-      </c>
-      <c r="D59" s="21" t="n">
-        <v>-0.1530551020408163</v>
-      </c>
-      <c r="E59" s="9" t="inlineStr">
-        <is>
-          <t>REDUCE</t>
-        </is>
+      <c r="C59" s="20">
+        <f>0.5*30*B59+0.3*28*B59+0.2*$B$28</f>
+        <v/>
+      </c>
+      <c r="D59" s="21">
+        <f>C59/1078-1+0.0047</f>
+        <v/>
+      </c>
+      <c r="E59" s="9">
+        <f>IF(D59&gt;$B$41,"BUY",IF(D59&gt;0.0882,"ACCUMULATE",IF(D59&gt;0,"HOLD","REDUCE")))</f>
+        <v/>
       </c>
     </row>
     <row r="60">
@@ -1683,16 +1695,17 @@
       <c r="B60" s="18" t="n">
         <v>33.1</v>
       </c>
-      <c r="C60" s="20" t="n">
-        <v>861</v>
-      </c>
-      <c r="D60" s="21" t="n">
-        <v>-0.1964688311688312</v>
-      </c>
-      <c r="E60" s="9" t="inlineStr">
-        <is>
-          <t>REDUCE</t>
-        </is>
+      <c r="C60" s="20">
+        <f>0.5*30*B60+0.3*28*B60+0.2*$B$28</f>
+        <v/>
+      </c>
+      <c r="D60" s="21">
+        <f>C60/1078-1+0.0047</f>
+        <v/>
+      </c>
+      <c r="E60" s="9">
+        <f>IF(D60&gt;$B$41,"BUY",IF(D60&gt;0.0882,"ACCUMULATE",IF(D60&gt;0,"HOLD","REDUCE")))</f>
+        <v/>
       </c>
     </row>
     <row r="62" ht="52" customHeight="1">
@@ -3003,7 +3016,7 @@
     <row r="30" ht="56" customHeight="1">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>A 55% spread between the highest and lowest target is extraordinary for a Nifty 50 constituent, and it tells you this is a genuinely contested stock rather than a mispriced one. Our ₹999 sits almost exactly on Emkay's ₹1,000, inside a bear cluster of five houses — and their stated reasoning is ours: rich valuation, questions over growth and return on equity, and funding-cost pressure. Bernstein: 'much of the positives are priced into the stock's rich valuations.' Macquarie: execution is good but 'valuation remains expensive' with rising borrowing costs a risk to margins.</t>
+          <t>A 55% spread between the highest and lowest target is extraordinary for a Nifty 50 constituent, and it tells you this is a genuinely contested stock rather than a mispriced one. Our ₹1,007 sits almost exactly on Emkay's ₹1,000, inside a bear cluster of five houses — and their stated reasoning is ours: rich valuation, questions over growth and return on equity, and funding-cost pressure. Bernstein: 'much of the positives are priced into the stock's rich valuations.' Macquarie: execution is good but 'valuation remains expensive' with rising borrowing costs a risk to margins.</t>
         </is>
       </c>
     </row>

</xml_diff>